<commit_message>
ui(pay): clearer sample buttons + replace fake addresses with placeholders
Two related changes addressing the same UX risk: an operator using
the sample as a starting point might forget to replace the example
data, then ship test addresses to production.

- Download buttons now read "↓ Sample CSV" and "↓ Sample Excel" so
  the affordance is unambiguous (the previous "↓ CSV / ↓ Excel" was
  too terse).
- Sample data is now placeholder-only: every cell reads
  "<input recipient address>", "<input amount>" etc. instead of
  Hardhat test addresses (0xf39Fd6e51..., etc.) that look real
  enough to land in production by accident. Uploading the unmodified
  sample now errors out cleanly with "Skipped 4 row(s) with
  malformed address" — exactly the safe failure mode.
- Comment header now leads with a "THIS IS A TEMPLATE" warning so
  the intent is obvious whether the user opens the file in a text
  editor or in Excel.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/pay/public/samples/recipients-sample.xlsx
+++ b/apps/pay/public/samples/recipients-sample.xlsx
@@ -16,25 +16,28 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
+    <t># THIS IS A TEMPLATE — replace every &lt;input ...&gt; placeholder below before uploading.</t>
+  </si>
+  <si>
+    <t># All addresses are intentionally invalid so an as-is upload errors out instead of</t>
+  </si>
+  <si>
+    <t># accidentally paying fictional accounts.</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
     <t># Amount is in the token you pick in the wizard (USDC / USDT / ETH / TON).</t>
   </si>
   <si>
-    <t># Optional 5th column `meta_address` — when filled, the system derives</t>
-  </si>
-  <si>
-    <t># a one-time stealth address per recipient automatically (privacy mode).</t>
-  </si>
-  <si>
-    <t># Leave it blank for a regular EOA payout. The example row below shows</t>
-  </si>
-  <si>
-    <t># the stealth case: address column empty, meta_address filled. REPLACE</t>
-  </si>
-  <si>
-    <t># the placeholder meta_address with the recipient's actual EIP-5564 key</t>
-  </si>
-  <si>
-    <t># (format: `st:eth:0x` + 132 hex chars).</t>
+    <t># Optional 5th column `meta_address` — when filled, the system derives a one-time</t>
+  </si>
+  <si>
+    <t># stealth address per recipient automatically (privacy mode). Leave blank for a</t>
+  </si>
+  <si>
+    <t># regular EOA payout. Format: `st:eth:0x` + 132 hex chars.</t>
   </si>
   <si>
     <t>name</t>
@@ -52,49 +55,28 @@
     <t>meta_address</t>
   </si>
   <si>
-    <t>Alice Kim</t>
-  </si>
-  <si>
-    <t>0xf39Fd6e51aad88F6F4ce6aB8827279cffFb92266</t>
-  </si>
-  <si>
-    <t>alice@example.com</t>
-  </si>
-  <si>
-    <t>Bob Lee</t>
-  </si>
-  <si>
-    <t>0x70997970C51812dc3A010C7d01b50e0d17dc79C8</t>
-  </si>
-  <si>
-    <t>bob@example.com</t>
-  </si>
-  <si>
-    <t>Carol Park</t>
-  </si>
-  <si>
-    <t>0x3C44CdDdB6a900fa2b585dd299e03d12FA4293BC</t>
-  </si>
-  <si>
-    <t>carol@example.com</t>
-  </si>
-  <si>
-    <t>Dave Stealth (replace meta_address)</t>
-  </si>
-  <si>
-    <t>dave@example.com</t>
-  </si>
-  <si>
-    <t>st:eth:0x03ebf948270e460d6dde0385f6fbc7d303d7fa6cbb9ce8a76ad23edbcd3e28c37d02afe23955ae8a9f4ef7d09a27c88f3ee7a45661d44ab526ed3d1832f35a2c95cb</t>
+    <t>&lt;input recipient name&gt;</t>
+  </si>
+  <si>
+    <t>&lt;input recipient address&gt;</t>
+  </si>
+  <si>
+    <t>&lt;input amount&gt;</t>
+  </si>
+  <si>
+    <t>&lt;input email&gt;</t>
+  </si>
+  <si>
+    <t>&lt;input stealth recipient name&gt;</t>
+  </si>
+  <si>
+    <t>&lt;input st:eth:0x... meta_address (or leave blank)&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="100" formatCode="0.00"/>
-  </numFmts>
   <fonts count="3">
     <font>
       <family val="2"/>
@@ -131,11 +113,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf/>
     <xf fontId="1" applyFont="1"/>
     <xf fontId="2" applyFont="1"/>
-    <xf numFmtId="100" applyNumberFormat="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -214,80 +195,89 @@
       <c r="E7" s="1"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
+      <c r="E9" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="3">
-        <v>3500</v>
-      </c>
-      <c r="D9" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3">
-        <v>3500</v>
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="3">
-        <v>4200</v>
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="3">
-        <v>5000</v>
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" t="s">
-        <v>23</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
@@ -295,6 +285,7 @@
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A8:E8"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ui(pay): sample CSV/Excel — one concrete example per mode
Two example rows so users see the column shape directly:

  1. Alice (sample — replace) → regular EOA, address = 0x000…000
  2. Bob Stealth (sample — replace) → stealth, address blank,
     meta_address = deterministic placeholder

Address column is intentionally the zero address: clearly not a real
recipient, and the wizard's review screen treats 0x0…0 as a burn
signal — much safer than the previous Hardhat test addresses
(0xf39Fd6e5…), which look real enough that a hurried operator could
ship them. Comment header now spells out exactly what each row is and
warns explicitly that 0x0 = burn.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/pay/public/samples/recipients-sample.xlsx
+++ b/apps/pay/public/samples/recipients-sample.xlsx
@@ -16,30 +16,30 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
-    <t># THIS IS A TEMPLATE — replace every &lt;input ...&gt; placeholder below before uploading.</t>
-  </si>
-  <si>
-    <t># All addresses are intentionally invalid so an as-is upload errors out instead of</t>
-  </si>
-  <si>
-    <t># accidentally paying fictional accounts.</t>
+    <t># THIS IS A TEMPLATE — replace every value below before uploading.</t>
+  </si>
+  <si>
+    <t># Addresses are 0x000…000 placeholders. Submitting them as-is would BURN funds.</t>
   </si>
   <si>
     <t>#</t>
   </si>
   <si>
+    <t># Row 1: regular EOA payout — replace `address`, `amount`, `email`, and `name`.</t>
+  </si>
+  <si>
+    <t># Row 2: stealth payout — leave `address` blank, replace `meta_address` with the</t>
+  </si>
+  <si>
+    <t># recipient's EIP-5564 key (format: `st:eth:0x` + 132 hex chars). The system</t>
+  </si>
+  <si>
+    <t># derives a one-time stealth address per recipient automatically.</t>
+  </si>
+  <si>
     <t># Amount is in the token you pick in the wizard (USDC / USDT / ETH / TON).</t>
   </si>
   <si>
-    <t># Optional 5th column `meta_address` — when filled, the system derives a one-time</t>
-  </si>
-  <si>
-    <t># stealth address per recipient automatically (privacy mode). Leave blank for a</t>
-  </si>
-  <si>
-    <t># regular EOA payout. Format: `st:eth:0x` + 132 hex chars.</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
@@ -55,28 +55,31 @@
     <t>meta_address</t>
   </si>
   <si>
-    <t>&lt;input recipient name&gt;</t>
-  </si>
-  <si>
-    <t>&lt;input recipient address&gt;</t>
-  </si>
-  <si>
-    <t>&lt;input amount&gt;</t>
-  </si>
-  <si>
-    <t>&lt;input email&gt;</t>
-  </si>
-  <si>
-    <t>&lt;input stealth recipient name&gt;</t>
-  </si>
-  <si>
-    <t>&lt;input st:eth:0x... meta_address (or leave blank)&gt;</t>
+    <t>Alice (sample — replace)</t>
+  </si>
+  <si>
+    <t>0x0000000000000000000000000000000000000000</t>
+  </si>
+  <si>
+    <t>alice@example.com</t>
+  </si>
+  <si>
+    <t>Bob Stealth (sample — replace)</t>
+  </si>
+  <si>
+    <t>bob@example.com</t>
+  </si>
+  <si>
+    <t>st:eth:0x03ebf948270e460d6dde0385f6fbc7d303d7fa6cbb9ce8a76ad23edbcd3e28c37d02afe23955ae8a9f4ef7d09a27c88f3ee7a45661d44ab526ed3d1832f35a2c95cb</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="100" formatCode="0.00"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <family val="2"/>
@@ -113,10 +116,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf/>
     <xf fontId="1" applyFont="1"/>
     <xf fontId="2" applyFont="1"/>
+    <xf numFmtId="100" applyNumberFormat="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -196,7 +200,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -204,34 +208,29 @@
       <c r="E8" s="1"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -241,43 +240,29 @@
       <c r="B11" t="s">
         <v>14</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3">
+        <v>100</v>
+      </c>
+      <c r="D11" t="s">
         <v>15</v>
-      </c>
-      <c r="D11" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="C12" s="3">
+        <v>100</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
         <v>17</v>
       </c>
-      <c r="C13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="E12" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
@@ -286,6 +271,7 @@
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>